<commit_message>
feat: enhance Excel processing with date handling and column style copying
</commit_message>
<xml_diff>
--- a/gdt-aggregated-xlsx/hd_sold_merged.xlsx
+++ b/gdt-aggregated-xlsx/hd_sold_merged.xlsx
@@ -6913,8 +6913,8 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7261,11 +7261,11 @@
     <col min="13" max="15" width="19.5" customWidth="1"/>
     <col min="16" max="17" width="11.6640625" customWidth="1"/>
     <col min="18" max="18" width="19.5" customWidth="1"/>
-    <col min="19" max="19" width="50.83203125" customWidth="1"/>
+    <col min="19" max="20" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="20:20" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="20:20" x14ac:dyDescent="0.25"/>
+    <row r="1" spans="19:20" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="19:20" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
@@ -7288,6 +7288,7 @@
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -7311,8 +7312,9 @@
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
-    </row>
-    <row r="5" spans="20:20" x14ac:dyDescent="0.25"/>
+      <c r="T4" s="2"/>
+    </row>
+    <row r="5" spans="19:20" x14ac:dyDescent="0.25"/>
     <row r="6" ht="50" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>2</v>
@@ -7371,7 +7373,7 @@
       <c r="S6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="T6" t="s">
+      <c r="T6" s="3" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>